<commit_message>
new pages added - ipo
</commit_message>
<xml_diff>
--- a/Database/Dashboard.xlsx
+++ b/Database/Dashboard.xlsx
@@ -449,18 +449,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SCI.NS</t>
+          <t>PNBHOUSING.NS</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>320</v>
+        <v>988</v>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20-04-2026 09:23:15</t>
+          <t>21-04-2026 13:50:56</t>
         </is>
       </c>
     </row>

</xml_diff>